<commit_message>
docs(NV3): add 5 Decision Table test cases TC-LOGIN-DT1..DT5 to test-cases.xlsx
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -547,7 +547,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -924,7 +923,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1128,7 +1126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1155,7 +1153,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1555,6 +1552,231 @@
       <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Giữ nguyên trang đăng nhập; hiển thị lỗi: 'Epic sadface: Username and password do not match any user in this service'</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-DT1</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Đăng nhập với Username và Password cùng để trống (Quy tắc R1)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>FR-01</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Bảng quyết định (DT)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Đang ở trang đăng nhập SauceDemo (https://www.saucedemo.com)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>user: ""
+pass: ""</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>1. Để trống Username
+2. Để trống Password
+3. Nhấn nút 'Login'</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Giữ nguyên trang đăng nhập; hiển thị thông báo lỗi: 'Epic sadface: Username is required'</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-DT2</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Đăng nhập đúng Username nhưng để trống Password (Quy tắc R2)</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>FR-01</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Bảng quyết định (DT)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Đang ở trang đăng nhập SauceDemo</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>user: standard_user
+pass: ""</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập Username 'standard_user'
+2. Để trống Password
+3. Nhấn nút 'Login'</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Giữ nguyên trang đăng nhập; hiển thị thông báo lỗi: 'Epic sadface: Password is required'</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-DT3</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Đăng nhập tài khoản bị khóa nhưng sai Password (Quy tắc R3)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>FR-01</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Bảng quyết định (DT)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Đang ở trang đăng nhập SauceDemo</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>user: locked_out_user
+pass: wrong_password</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập Username 'locked_out_user'
+2. Nhập Password 'wrong_password'
+3. Nhấn nút 'Login'</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Giữ nguyên trang đăng nhập; hiển thị thông báo lỗi: 'Epic sadface: Username and password do not match any user in this service'</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-DT4</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Đăng nhập tài khoản bị khóa với đúng Password (Quy tắc R4)</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>FR-01</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Bảng quyết định (DT)</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Đang ở trang đăng nhập SauceDemo</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>user: locked_out_user
+pass: secret_sauce</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập Username 'locked_out_user'
+2. Nhập Password 'secret_sauce'
+3. Nhấn nút 'Login'</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Giữ nguyên trang đăng nhập; hiển thị thông báo lỗi: 'Epic sadface: Sorry, this user has been locked out.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-DT5</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công với tài khoản và Password đúng (Quy tắc R5)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>FR-01</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Bảng quyết định (DT)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Đang ở trang đăng nhập SauceDemo</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>user: standard_user
+pass: secret_sauce</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>1. Nhập Username 'standard_user'
+2. Nhập Password 'secret_sauce'
+3. Nhấn nút 'Login'</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công, chuyển hướng đến trang 'inventory.html'</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1818,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2056,7 +2277,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(Excel): sync Requirements sheet with detailed member specifications
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -572,12 +572,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Đăng nhập thành công với tài khoản hợp lệ (standard_user / secret_sauce)</t>
+          <t>Đăng nhập thành công với tài khoản hợp lệ</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Chuyển hướng sang trang danh sách sản phẩm với URL: https://www.saucedemo.com/inventory.html</t>
+          <t>Nhập standard_user / secret_sauce -&gt; Chuyển hướng sang URL https://www.saucedemo.com/inventory.html</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Giữ nguyên tại trang đăng nhập; hiển thị thông báo lỗi: "Epic sadface: Username is required"</t>
+          <t>Bỏ trống username -&gt; Giữ nguyên trang đăng nhập; hiển thị lỗi: "Epic sadface: Username is required"</t>
         </is>
       </c>
     </row>
@@ -606,12 +606,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra để trống trường Password khi đã nhập Username</t>
+          <t>Kiểm tra để trống trường Password</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Giữ nguyên tại trang đăng nhập; hiển thị thông báo lỗi: "Epic sadface: Password is required"</t>
+          <t>Có username nhưng để trống password -&gt; Giữ nguyên trang đăng nhập; hiển thị lỗi: "Epic sadface: Password is required"</t>
         </is>
       </c>
     </row>
@@ -623,12 +623,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Kiểm tra thông tin đăng nhập không hợp lệ (sai username, sai password, hoặc sai chữ hoa/thường)</t>
+          <t>Kiểm tra thông tin sai hoặc sai chữ hoa/thường</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Giữ nguyên tại trang đăng nhập; hiển thị thông báo lỗi: "Epic sadface: Username and password do not match any user in this service"</t>
+          <t>Nhập sai tên, sai mật khẩu, hoặc sai chữ hoa/thường -&gt; Hiển thị lỗi: "Epic sadface: Username and password do not match any user in this service"</t>
         </is>
       </c>
     </row>
@@ -640,12 +640,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Đăng nhập bằng tài khoản bị khóa (locked_out_user / secret_sauce)</t>
+          <t>Đăng nhập tài khoản bị khóa</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Giữ nguyên tại trang đăng nhập; hiển thị thông báo lỗi: "Epic sadface: Sorry, this user has been locked out."</t>
+          <t>Nhập locked_out_user / secret_sauce -&gt; Hiển thị lỗi: "Epic sadface: Sorry, this user has been locked out."</t>
         </is>
       </c>
     </row>
@@ -657,12 +657,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Thêm sản phẩm vào giỏ hàng từ trang sản phẩm (inventory.html)</t>
+          <t>Trạng thái nút Add to cart</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Nút "Add to cart" đổi thành "Remove"; Badge hiển thị số lượng sản phẩm (1-6) tương ứng</t>
+          <t>Sản phẩm chưa được thêm vào giỏ sẽ hiển thị nút "Add to cart". Khi người dùng nhấn nút này, sản phẩm được thêm vào giỏ; hiện thêm nút "Remove" trong giỏ hàng và badge tăng thêm 1.</t>
         </is>
       </c>
     </row>
@@ -674,216 +674,267 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Xóa sản phẩm khỏi giỏ hàng từ trang sản phẩm hoặc trang giỏ hàng (cart.html)</t>
+          <t>Trạng thái nút Remove</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Nút "Remove" đổi thành "Add to cart"; Badge giảm tương ứng; khi giỏ hàng rỗng thì Badge biến mất hoàn toàn</t>
+          <t>Khi người dùng nhấn nút "Remove", sản phẩm tương ứng bị xóa khỏi giỏ; nút đổi trở lại "Add to cart" và badge giảm đi 1.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>FR-03.1</t>
+          <t>FR-02.3</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Kiểm tra First Name bắt buộc tại bước thanh toán (checkout-step-one.html)</t>
+          <t>Badge hiển thị số lượng từ 1 đến 6</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Không được để trống. Nếu First Name rỗng -&gt; hiển thị lỗi: "Error: First Name is required"</t>
+          <t>Khi giỏ có từ 1 đến 6 sản phẩm, badge hiển thị đúng số lượng sản phẩm hiện có. Ví dụ: có 3 sản phẩm thì badge hiển thị số 3; có đủ 6 sản phẩm thì badge hiển thị số 6.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>FR-03.2</t>
+          <t>FR-02.4</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Kiểm tra Last Name bắt buộc tại bước thanh toán</t>
+          <t>Giỏ hàng rỗng</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Nếu First Name hợp lệ nhưng Last Name rỗng -&gt; hiển thị lỗi: "Error: Last Name is required"</t>
+          <t>Khi chưa có sản phẩm nào được thêm vào giỏ hoặc khi tất cả sản phẩm đã bị xóa, badge không hiển thị (ẩn hoàn toàn). Các sản phẩm đã bị xóa hiển thị lại nút "Add to cart".</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>FR-03.3</t>
+          <t>FR-03.1</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Kiểm tra Postal Code bắt buộc tại bước thanh toán</t>
+          <t>Kiểm tra First Name</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Nếu First Name và Last Name hợp lệ nhưng Postal Code rỗng -&gt; hiển thị lỗi: "Error: Postal Code is required"</t>
+          <t>Không được để trống; Nếu để trống hiển thị Error: First Name is required</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>FR-03.4</t>
+          <t>FR-03.2</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Tính tiền thuế (Tax) tại bước tổng quan (checkout-step-two.html)</t>
+          <t>Kiểm tra Last Name</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Tiền thuế hiển thị theo công thức: Tax = 8% * Item total (làm tròn đến 2 chữ số thập phân)</t>
+          <t>Nếu First name hợp lệ nhưng Last Name trống hiển thị Error: Last Name is required</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>FR-03.5</t>
+          <t>FR-03.3</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Tính tổng thanh toán (Total) tại bước tổng quan</t>
+          <t>Kiểm tra Postal Code</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Tổng tiền thanh toán hiển thị theo công thức: Total = Item total + Tax</t>
+          <t>Nếu cả 2 trường hợp First và Last Name đều hợp lệ nhưng Postal Code để trống hiển thị Error: Postal Code is required</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>FR-03.6</t>
+          <t>FR-03.4</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Hoàn tất đơn hàng (Finish) tại trang checkout-complete.html</t>
+          <t>Tính tiền thuế</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Chuyển đến checkout-complete.html, hiển thị: "Thank you for your order!", giỏ hàng được làm rỗng và Badge biến mất</t>
+          <t>Tax bằng 8% Item Total, làm tròn đến 2 chữ số thập phân</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>FR-03.7</t>
+          <t>FR-03.5</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Hủy bỏ thanh toán (Cancel) tại bước nhập thông tin</t>
+          <t>Tính tổng thanh toán</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Nhấn nút Cancel chuyển hướng quay về URL cart.html, các sản phẩm đã chọn vẫn còn nguyên trong giỏ hàng</t>
+          <t>Tổng tiền sẽ bằng cho giá sản phẩm cộng thêm giá tiền thuế: Total = Item Total + Tax</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>FR-04.1</t>
+          <t>FR-03.6</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Sắp xếp sản phẩm theo tên A to Z</t>
+          <t>Hoàn tất đơn hàng</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Danh sách sản phẩm được sắp xếp theo thứ tự bảng chữ cái tăng dần của tên sản phẩm</t>
+          <t>Hiển thị Thank you for your order! và giỏ hàng được làm trống</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>FR-04.2</t>
+          <t>FR-03.7</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Sắp xếp sản phẩm theo tên Z to A</t>
+          <t>Hủy tại bước nhập thông tin</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Danh sách sản phẩm được sắp xếp theo thứ tự bảng chữ cái giảm dần của tên sản phẩm</t>
+          <t>Chuyển về cart.html các sản phẩm đã chọn vẫn còn nguyên trong giỏ hàng</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>FR-04.3</t>
+          <t>FR-04.1</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Sắp xếp sản phẩm theo giá Low to High</t>
+          <t>Sắp xếp theo Name (A to Z)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Danh sách sản phẩm được sắp xếp theo giá tăng dần ($7.99 -&gt; $49.99)</t>
+          <t>Sắp xếp sản phẩm theo thứ tự bảng chữ cái tăng dần A-Z. Nếu trùng các chữ cái đầu, so sánh ký tự tiếp theo. Với 3 sản phẩm mẫu: Sauce Labs Backpack, Sauce Labs Bike Light, Sauce Labs Bolt T-Shirt -&gt; Hiển thị đúng thứ tự: Backpack -&gt; Bike Light -&gt; Bolt T-Shirt</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>FR-04.4</t>
+          <t>FR-04.2</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Sắp xếp sản phẩm theo giá High to Low</t>
+          <t>Sắp xếp theo Name (Z to A)</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Danh sách sản phẩm được sắp xếp theo giá giảm dần ($49.99 -&gt; $7.99)</t>
+          <t>Sắp xếp sản phẩm theo thứ tự bảng chữ cái giảm dần Z-A. Nếu trùng các chữ cái đầu, so sánh ký tự tiếp theo. Với 3 sản phẩm trên -&gt; Hiển thị đảo ngược: Bolt T-Shirt -&gt; Bike Light -&gt; Backpack</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>NFR-01</t>
+          <t>FR-04.3</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Hiệu năng tải trang sản phẩm sau khi đăng nhập đúng</t>
+          <t>Sắp xếp theo Price (low to high)</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Sau khi nhấn Login với thông tin đúng, trang sản phẩm (inventory.html) phải hiển thị trong tối đa 3 giây (trung vị của 5 lần đo, mạng ổn định)</t>
+          <t>Sắp xếp sản phẩm theo giá từ thấp tới cao. Sản phẩm đầu danh sách có giá thấp nhất là $7.99 (Sauce Labs Onesie), sản phẩm cuối cùng có giá cao nhất là $49.99 (Sauce Labs Fleece Jacket). Giá phía trên luôn &lt;= giá liền kề phía dưới.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>FR-04.4</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Sắp xếp theo Price (high to low)</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Sắp xếp sản phẩm theo giá từ cao tới thấp. Sản phẩm đầu danh sách có giá cao nhất là $49.99 (Sauce Labs Fleece Jacket), sản phẩm cuối cùng có giá thấp nhất là $7.99 (Sauce Labs Onesie). Giá phía trên luôn &gt;= giá liền kề phía dưới.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>NFR-01.1</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Tiêu chuẩn thời gian hiển thị trang sản phẩm</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Khi người dùng nhập đúng thông tin đăng nhập và nhấn nút Login, hệ thống phải hiển thị trang danh sách sản phẩm trong thời gian không vượt quá 3 giây. Tiêu chí chấp nhận: Trung vị thời gian đo &lt;= 3.000 ms (3s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>NFR-01.2</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Điều kiện và phương pháp đo kiểm</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Tài khoản: performance_glitch_user, mật khẩu: secret_sauce, mạng ổn định. Thực hiện 5 lần đo độc lập, ghi nhận từ khi nhấn Login đến khi trang inventory.html hiển thị hoàn tất, tính trung vị 5 lần.</t>
         </is>
       </c>
     </row>

</xml_diff>